<commit_message>
Before big death change
</commit_message>
<xml_diff>
--- a/data/tier_app/iedea_indicators/indicator_artstart.xlsx
+++ b/data/tier_app/iedea_indicators/indicator_artstart.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2ae90f5cbd0fd171/AMC/HIV Prioritization tool/HIV_prioritization_tool/data/tier_app/iedea_indicators/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{22C88673-57F5-B04B-8EE2-642DDA56B525}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{B3F86211-B80C-D540-984E-5C44C2DFF56C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-33700" yWindow="-960" windowWidth="27640" windowHeight="15320" activeTab="1" xr2:uid="{0A9E637F-422C-BE40-81DF-DED3F7B193D2}"/>
+    <workbookView xWindow="-34820" yWindow="-1140" windowWidth="33980" windowHeight="19140" activeTab="1" xr2:uid="{0A9E637F-422C-BE40-81DF-DED3F7B193D2}"/>
   </bookViews>
   <sheets>
     <sheet name="indicator_artstart" sheetId="1" r:id="rId1"/>
@@ -39,8 +39,108 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:xdr="http://purl.oclc.org/ooxml/drawingml/spreadsheetDrawing" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Leigh Johnson</author>
+  </authors>
+  <commentList>
+    <comment ref="A45" authorId="0" shapeId="2051" xr:uid="{C7F5560C-5891-0D4A-8B02-151CE51B31CA}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Leigh Johnson:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Parameters are specified for age 30.</t>
+        </r>
+      </text>
+      <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+        <mc:Choice Requires="v"/>
+        <mc:Fallback>
+          <commentPr defaultSize="0" autoFill="0" autoLine="0">
+            <anchor>
+              <from>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>190500</xdr:colOff>
+                <xdr:row>43</xdr:row>
+                <xdr:rowOff>76200</xdr:rowOff>
+              </from>
+              <to>
+                <xdr:col>2</xdr:col>
+                <xdr:colOff>711200</xdr:colOff>
+                <xdr:row>46</xdr:row>
+                <xdr:rowOff>190500</xdr:rowOff>
+              </to>
+            </anchor>
+          </commentPr>
+        </mc:Fallback>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="A51" authorId="0" shapeId="2052" xr:uid="{68A8BE86-5723-0548-9CD5-6D29C09EDB43}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Leigh Johnson:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Parameters are specified for age 30.</t>
+        </r>
+      </text>
+      <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+        <mc:Choice Requires="v"/>
+        <mc:Fallback>
+          <commentPr defaultSize="0" autoFill="0" autoLine="0">
+            <anchor>
+              <from>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>190500</xdr:colOff>
+                <xdr:row>49</xdr:row>
+                <xdr:rowOff>76200</xdr:rowOff>
+              </from>
+              <to>
+                <xdr:col>2</xdr:col>
+                <xdr:colOff>711200</xdr:colOff>
+                <xdr:row>52</xdr:row>
+                <xdr:rowOff>190500</xdr:rowOff>
+              </to>
+            </anchor>
+          </commentPr>
+        </mc:Fallback>
+      </mc:AlternateContent>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="5076" uniqueCount="65">
+<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="5096" uniqueCount="84">
   <si>
     <t>Region</t>
   </si>
@@ -243,9 +343,6 @@
     <t>&lt;50</t>
   </si>
   <si>
-    <t>Annual mortality</t>
-  </si>
-  <si>
     <t>Avg</t>
   </si>
   <si>
@@ -257,12 +354,75 @@
   <si>
     <t>200-350</t>
   </si>
+  <si>
+    <t>&lt;200</t>
+  </si>
+  <si>
+    <t>Annual mortality no on treatment</t>
+  </si>
+  <si>
+    <t>Weighted average 350+</t>
+  </si>
+  <si>
+    <t>Prop 350+</t>
+  </si>
+  <si>
+    <t>Thembisa mortality</t>
+  </si>
+  <si>
+    <t>CD4 stage at ART initiation</t>
+  </si>
+  <si>
+    <t>350-499</t>
+  </si>
+  <si>
+    <t>200-349</t>
+  </si>
+  <si>
+    <t>Annual HIV mortality rate during first 6 months of ART, males</t>
+  </si>
+  <si>
+    <t>Annual HIV mortality rate during first months 7-18 of ART, males</t>
+  </si>
+  <si>
+    <t>Annual HIV mortality rate during first 19-30 months of ART, males</t>
+  </si>
+  <si>
+    <t>Annual HIV mortality rate during first 31-42 months of ART, males</t>
+  </si>
+  <si>
+    <t>Annual HIV mortality rate after first 42 months of ART, males</t>
+  </si>
+  <si>
+    <t>Annual HIV mortality rate during first 6 months of ART, females</t>
+  </si>
+  <si>
+    <t>Annual HIV mortality rate during first months 7-18 of ART, females</t>
+  </si>
+  <si>
+    <t>Annual HIV mortality rate during first 19-30 months of ART, females</t>
+  </si>
+  <si>
+    <t>Annual HIV mortality rate during first 31-42 months of ART, females</t>
+  </si>
+  <si>
+    <t>Annual HIV mortality rate after first 42 months of ART, females</t>
+  </si>
+  <si>
+    <t>Take 0.0045 for treated suppressed and unsurpressed non-AHD established</t>
+  </si>
+  <si>
+    <t>Untreataed AHD take 0.18 (first 6 months)</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="20" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="167" formatCode="0.0000"/>
+  </numFmts>
+  <fonts count="24" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -409,6 +569,30 @@
       <color rgb="FF1B1B1B"/>
       <name val="Cambria"/>
       <family val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="33">
@@ -752,9 +936,12 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="9" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -859,6 +1046,222 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:v="urn:schemas-microsoft-com:vml" Requires="v"/>
+    <mc:Fallback>
+      <xdr:twoCellAnchor editAs="absolute">
+        <xdr:from>
+          <xdr:col>1</xdr:col>
+          <xdr:colOff>190500</xdr:colOff>
+          <xdr:row>43</xdr:row>
+          <xdr:rowOff>76200</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>2</xdr:col>
+          <xdr:colOff>711200</xdr:colOff>
+          <xdr:row>46</xdr:row>
+          <xdr:rowOff>190500</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="2051" name="Comment 3" hidden="1">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{706079A3-6B1E-4428-B605-29BE2DBB932F}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr txBox="1">
+              <a:spLocks noChangeArrowheads="1"/>
+            </xdr:cNvSpPr>
+          </xdr:nvSpPr>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="1016000" y="9601200"/>
+              <a:ext cx="1346200" cy="723900"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:srgbClr val="FFFFE1"/>
+            </a:solidFill>
+            <a:ln w="9525">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:miter lim="800%"/>
+              <a:headEnd/>
+              <a:tailEnd/>
+            </a:ln>
+            <a:effectLst>
+              <a:outerShdw dist="35921" dir="2700000" algn="ctr" rotWithShape="0">
+                <a:srgbClr val="000000"/>
+              </a:outerShdw>
+            </a:effectLst>
+            <a:extLst>
+              <a:ext uri="{53640926-AAD7-44D8-BBD7-CCE9431645EC}">
+                <a14:shadowObscured xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="1"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" wrap="square" lIns="27432" tIns="18288" rIns="0" bIns="0" anchor="t" upright="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr algn="l" rtl="0">
+                <a:defRPr sz="1000"/>
+              </a:pPr>
+              <a:r>
+                <a:rPr lang="en-GB" sz="800" b="1" i="0" u="none" strike="noStrike" baseline="0%">
+                  <a:solidFill>
+                    <a:srgbClr val="000000"/>
+                  </a:solidFill>
+                  <a:latin typeface="Tahoma" pitchFamily="2" charset="0"/>
+                  <a:ea typeface="Tahoma" pitchFamily="2" charset="0"/>
+                  <a:cs typeface="Tahoma" pitchFamily="2" charset="0"/>
+                </a:rPr>
+                <a:t>Leigh Johnson:</a:t>
+              </a:r>
+              <a:endParaRPr lang="en-GB" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0%">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Tahoma" pitchFamily="2" charset="0"/>
+                <a:ea typeface="Tahoma" pitchFamily="2" charset="0"/>
+                <a:cs typeface="Tahoma" pitchFamily="2" charset="0"/>
+              </a:endParaRPr>
+            </a:p>
+            <a:p>
+              <a:pPr algn="l" rtl="0">
+                <a:defRPr sz="1000"/>
+              </a:pPr>
+              <a:r>
+                <a:rPr lang="en-GB" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0%">
+                  <a:solidFill>
+                    <a:srgbClr val="000000"/>
+                  </a:solidFill>
+                  <a:latin typeface="Tahoma" pitchFamily="2" charset="0"/>
+                  <a:ea typeface="Tahoma" pitchFamily="2" charset="0"/>
+                  <a:cs typeface="Tahoma" pitchFamily="2" charset="0"/>
+                </a:rPr>
+                <a:t>Parameters are specified for age 30.</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+        <xdr:clientData/>
+      </xdr:twoCellAnchor>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:v="urn:schemas-microsoft-com:vml" Requires="v"/>
+    <mc:Fallback>
+      <xdr:twoCellAnchor editAs="absolute">
+        <xdr:from>
+          <xdr:col>1</xdr:col>
+          <xdr:colOff>190500</xdr:colOff>
+          <xdr:row>49</xdr:row>
+          <xdr:rowOff>76200</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>2</xdr:col>
+          <xdr:colOff>711200</xdr:colOff>
+          <xdr:row>52</xdr:row>
+          <xdr:rowOff>190500</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="2052" name="Comment 4" hidden="1">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DB53D83D-75EE-93CE-42D1-8FFF8B8DA461}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr txBox="1">
+              <a:spLocks noChangeArrowheads="1"/>
+            </xdr:cNvSpPr>
+          </xdr:nvSpPr>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="1016000" y="10820400"/>
+              <a:ext cx="1346200" cy="723900"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:srgbClr val="FFFFE1"/>
+            </a:solidFill>
+            <a:ln w="9525">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:miter lim="800%"/>
+              <a:headEnd/>
+              <a:tailEnd/>
+            </a:ln>
+            <a:effectLst>
+              <a:outerShdw dist="35921" dir="2700000" algn="ctr" rotWithShape="0">
+                <a:srgbClr val="000000"/>
+              </a:outerShdw>
+            </a:effectLst>
+            <a:extLst>
+              <a:ext uri="{53640926-AAD7-44D8-BBD7-CCE9431645EC}">
+                <a14:shadowObscured xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="1"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" wrap="square" lIns="27432" tIns="18288" rIns="0" bIns="0" anchor="t" upright="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr algn="l" rtl="0">
+                <a:defRPr sz="1000"/>
+              </a:pPr>
+              <a:r>
+                <a:rPr lang="en-GB" sz="800" b="1" i="0" u="none" strike="noStrike" baseline="0%">
+                  <a:solidFill>
+                    <a:srgbClr val="000000"/>
+                  </a:solidFill>
+                  <a:latin typeface="Tahoma" pitchFamily="2" charset="0"/>
+                  <a:ea typeface="Tahoma" pitchFamily="2" charset="0"/>
+                  <a:cs typeface="Tahoma" pitchFamily="2" charset="0"/>
+                </a:rPr>
+                <a:t>Leigh Johnson:</a:t>
+              </a:r>
+              <a:endParaRPr lang="en-GB" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0%">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Tahoma" pitchFamily="2" charset="0"/>
+                <a:ea typeface="Tahoma" pitchFamily="2" charset="0"/>
+                <a:cs typeface="Tahoma" pitchFamily="2" charset="0"/>
+              </a:endParaRPr>
+            </a:p>
+            <a:p>
+              <a:pPr algn="l" rtl="0">
+                <a:defRPr sz="1000"/>
+              </a:pPr>
+              <a:r>
+                <a:rPr lang="en-GB" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0%">
+                  <a:solidFill>
+                    <a:srgbClr val="000000"/>
+                  </a:solidFill>
+                  <a:latin typeface="Tahoma" pitchFamily="2" charset="0"/>
+                  <a:ea typeface="Tahoma" pitchFamily="2" charset="0"/>
+                  <a:cs typeface="Tahoma" pitchFamily="2" charset="0"/>
+                </a:rPr>
+                <a:t>Parameters are specified for age 30.</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+        <xdr:clientData/>
+      </xdr:twoCellAnchor>
+    </mc:Fallback>
+  </mc:AlternateContent>
 </xdr:wsDr>
 </file>
 
@@ -93584,8 +93987,8 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C7501CA-F35A-1449-8DEB-8BD038E5B763}">
-  <dimension ref="A1:I38"/>
+<worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:xdr="http://purl.oclc.org/ooxml/drawingml/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C7501CA-F35A-1449-8DEB-8BD038E5B763}">
+  <dimension ref="A1:N55"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.2">
@@ -93816,6 +94219,9 @@
       <c r="E15" t="s">
         <v>45</v>
       </c>
+      <c r="F15" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B16" t="s">
@@ -93830,7 +94236,7 @@
         <v>0.35853410874180747</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B17" t="s">
         <v>41</v>
       </c>
@@ -93847,7 +94253,7 @@
         <v>0.34983450856238307</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B18" t="s">
         <v>42</v>
       </c>
@@ -93863,8 +94269,12 @@
         <f>C18/C22</f>
         <v>0.26449848899122175</v>
       </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F18">
+        <f>C18/(C18+C19)</f>
+        <v>0.40681717574147852</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B19" t="s">
         <v>43</v>
       </c>
@@ -93880,14 +94290,18 @@
         <f>C19/C22</f>
         <v>0.38566700244639518</v>
       </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F19">
+        <f>1-F18</f>
+        <v>0.59318282425852153</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="C20">
         <f>SUM(C16:C19)</f>
         <v>10833</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B22" t="s">
         <v>46</v>
       </c>
@@ -93896,17 +94310,17 @@
         <v>6949</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" ht="22" x14ac:dyDescent="0.25">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" ht="22" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="31" spans="1:9" ht="24" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" ht="24" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>48</v>
       </c>
@@ -93923,13 +94337,13 @@
         <v>52</v>
       </c>
       <c r="F31" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="H31" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="H31" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9" ht="22" x14ac:dyDescent="0.25">
+    </row>
+    <row r="32" spans="1:11" ht="22" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>53</v>
       </c>
@@ -93950,14 +94364,17 @@
         <v>4.7500000000000007E-3</v>
       </c>
       <c r="H32" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I32">
         <f>F32</f>
         <v>4.7500000000000007E-3</v>
       </c>
-    </row>
-    <row r="33" spans="1:9" ht="22" x14ac:dyDescent="0.25">
+      <c r="K32" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="33" spans="1:14" ht="22" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>54</v>
       </c>
@@ -93984,8 +94401,12 @@
         <f>F33</f>
         <v>1.1749999999999998E-2</v>
       </c>
-    </row>
-    <row r="34" spans="1:9" ht="22" x14ac:dyDescent="0.25">
+      <c r="K33">
+        <f>F32*F19+F33*F18</f>
+        <v>7.5977202301903499E-3</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14" ht="22" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>55</v>
       </c>
@@ -94006,14 +94427,14 @@
         <v>0.03</v>
       </c>
       <c r="H34" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="I34">
         <f>(2*F34+F35)/3</f>
         <v>4.5500000000000006E-2</v>
       </c>
     </row>
-    <row r="35" spans="1:9" ht="22" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:14" ht="22" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>56</v>
       </c>
@@ -94035,7 +94456,7 @@
       </c>
       <c r="H35" s="1"/>
     </row>
-    <row r="36" spans="1:9" ht="22" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:14" ht="22" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>57</v>
       </c>
@@ -94056,7 +94477,7 @@
         <v>0.19625000000000004</v>
       </c>
     </row>
-    <row r="37" spans="1:9" ht="22" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:14" ht="22" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>58</v>
       </c>
@@ -94077,7 +94498,7 @@
         <v>0.50600000000000001</v>
       </c>
     </row>
-    <row r="38" spans="1:9" ht="22" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:14" ht="22" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>59</v>
       </c>
@@ -94098,8 +94519,288 @@
         <v>1.3062499999999999</v>
       </c>
     </row>
+    <row r="41" spans="1:14" ht="22" x14ac:dyDescent="0.25">
+      <c r="A41" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="43" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A43" s="2"/>
+      <c r="G43" s="3" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="44" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A44" s="2"/>
+      <c r="G44" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="H44" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="I44" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="J44" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="K44" s="2"/>
+      <c r="L44" s="2"/>
+      <c r="M44" s="2"/>
+    </row>
+    <row r="45" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A45" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="G45" s="4">
+        <v>2.0000000000000001E-4</v>
+      </c>
+      <c r="H45" s="4">
+        <v>1.6000000000000001E-3</v>
+      </c>
+      <c r="I45" s="4">
+        <v>1.46E-2</v>
+      </c>
+      <c r="J45" s="4">
+        <v>0.21679999999999999</v>
+      </c>
+      <c r="K45" s="4"/>
+      <c r="L45" s="4">
+        <f>G45*E19+H45*E18+I45*E17</f>
+        <v>5.6079148078860266E-3</v>
+      </c>
+      <c r="M45" s="4"/>
+      <c r="N45" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="46" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A46" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="G46" s="4">
+        <v>8.9999999999999998E-4</v>
+      </c>
+      <c r="H46" s="4">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="I46" s="4">
+        <v>1.32E-2</v>
+      </c>
+      <c r="J46" s="4">
+        <v>5.33E-2</v>
+      </c>
+      <c r="K46" s="4"/>
+      <c r="L46" s="4">
+        <f>G46*$E$19+H46*$E$18+I46*$E$17</f>
+        <v>6.2874082601813205E-3</v>
+      </c>
+      <c r="M46" s="4"/>
+    </row>
+    <row r="47" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A47" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="G47" s="4">
+        <v>2.7000000000000001E-3</v>
+      </c>
+      <c r="H47" s="4">
+        <v>8.5000000000000006E-3</v>
+      </c>
+      <c r="I47" s="4">
+        <v>1.1599999999999999E-2</v>
+      </c>
+      <c r="J47" s="4">
+        <v>2.81E-2</v>
+      </c>
+      <c r="K47" s="4"/>
+      <c r="L47" s="4">
+        <f>G47*$E$19+H47*$E$18+I47*$E$17</f>
+        <v>7.3476183623542952E-3</v>
+      </c>
+      <c r="M47" s="4"/>
+    </row>
+    <row r="48" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A48" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="G48" s="4">
+        <v>4.1999999999999997E-3</v>
+      </c>
+      <c r="H48" s="4">
+        <v>7.6E-3</v>
+      </c>
+      <c r="I48" s="4">
+        <v>7.6E-3</v>
+      </c>
+      <c r="J48" s="4">
+        <v>1.8499999999999999E-2</v>
+      </c>
+      <c r="K48" s="4"/>
+      <c r="L48" s="4">
+        <f t="shared" ref="L48:L55" si="3">G48*$E$19+H48*$E$18+I48*$E$17</f>
+        <v>6.288732191682256E-3</v>
+      </c>
+      <c r="M48" s="4"/>
+    </row>
+    <row r="49" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A49" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="G49" s="4">
+        <v>4.8999999999999998E-3</v>
+      </c>
+      <c r="H49" s="4">
+        <v>6.3E-3</v>
+      </c>
+      <c r="I49" s="4">
+        <v>6.3E-3</v>
+      </c>
+      <c r="J49" s="4">
+        <v>1.52E-2</v>
+      </c>
+      <c r="K49" s="4"/>
+      <c r="L49" s="4">
+        <f t="shared" si="3"/>
+        <v>5.7600661965750474E-3</v>
+      </c>
+      <c r="M49" s="4"/>
+      <c r="N49" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="50" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A50" s="2"/>
+      <c r="G50" s="4"/>
+      <c r="H50" s="4"/>
+      <c r="I50" s="4"/>
+      <c r="J50" s="4"/>
+      <c r="K50" s="4"/>
+      <c r="L50" s="4"/>
+      <c r="M50" s="4"/>
+    </row>
+    <row r="51" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A51" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="G51" s="4">
+        <v>1E-4</v>
+      </c>
+      <c r="H51" s="4">
+        <v>1.6000000000000001E-3</v>
+      </c>
+      <c r="I51" s="4">
+        <v>1.5900000000000001E-2</v>
+      </c>
+      <c r="J51" s="4">
+        <v>0.1699</v>
+      </c>
+      <c r="K51" s="4"/>
+      <c r="L51" s="4">
+        <f t="shared" si="3"/>
+        <v>6.0241329687724856E-3</v>
+      </c>
+      <c r="M51" s="4"/>
+    </row>
+    <row r="52" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A52" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="G52" s="4">
+        <v>8.0000000000000004E-4</v>
+      </c>
+      <c r="H52" s="4">
+        <v>4.4999999999999997E-3</v>
+      </c>
+      <c r="I52" s="4">
+        <v>1.01E-2</v>
+      </c>
+      <c r="J52" s="4">
+        <v>4.1599999999999998E-2</v>
+      </c>
+      <c r="K52" s="4"/>
+      <c r="L52" s="4">
+        <f t="shared" si="3"/>
+        <v>5.0321053388976827E-3</v>
+      </c>
+      <c r="M52" s="4"/>
+    </row>
+    <row r="53" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A53" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="G53" s="4">
+        <v>2E-3</v>
+      </c>
+      <c r="H53" s="4">
+        <v>5.7000000000000002E-3</v>
+      </c>
+      <c r="I53" s="4">
+        <v>5.7000000000000002E-3</v>
+      </c>
+      <c r="J53" s="4">
+        <v>2.1600000000000001E-2</v>
+      </c>
+      <c r="K53" s="4"/>
+      <c r="L53" s="4">
+        <f t="shared" si="3"/>
+        <v>4.2730320909483378E-3</v>
+      </c>
+      <c r="M53" s="4"/>
+    </row>
+    <row r="54" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A54" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="G54" s="4">
+        <v>2.7000000000000001E-3</v>
+      </c>
+      <c r="H54" s="4">
+        <v>3.3999999999999998E-3</v>
+      </c>
+      <c r="I54" s="4">
+        <v>3.3999999999999998E-3</v>
+      </c>
+      <c r="J54" s="4">
+        <v>1.2999999999999999E-2</v>
+      </c>
+      <c r="K54" s="4"/>
+      <c r="L54" s="4">
+        <f t="shared" si="3"/>
+        <v>3.130033098287523E-3</v>
+      </c>
+      <c r="M54" s="4"/>
+    </row>
+    <row r="55" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A55" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="G55" s="4">
+        <v>2.5000000000000001E-3</v>
+      </c>
+      <c r="H55" s="4">
+        <v>2.5000000000000001E-3</v>
+      </c>
+      <c r="I55" s="4">
+        <v>2.5000000000000001E-3</v>
+      </c>
+      <c r="J55" s="4">
+        <v>9.4000000000000004E-3</v>
+      </c>
+      <c r="K55" s="4"/>
+      <c r="L55" s="4">
+        <f>G55*$E$19+H55*$E$18+I55*$E$17</f>
+        <v>2.5000000000000001E-3</v>
+      </c>
+      <c r="M55" s="4"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="v">
+      <legacyDrawing r:id="rId2"/>
+    </mc:Choice>
+  </mc:AlternateContent>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Mortality calibration and retest prop changes
</commit_message>
<xml_diff>
--- a/data/tier_app/iedea_indicators/indicator_artstart.xlsx
+++ b/data/tier_app/iedea_indicators/indicator_artstart.xlsx
@@ -8,18 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2ae90f5cbd0fd171/AMC/HIV Prioritization tool/HIV_prioritization_tool/data/tier_app/iedea_indicators/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{B3F86211-B80C-D540-984E-5C44C2DFF56C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{5F580FA2-E213-384C-BADC-BD5F5FA04472}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-34820" yWindow="-1140" windowWidth="33980" windowHeight="19140" activeTab="1" xr2:uid="{0A9E637F-422C-BE40-81DF-DED3F7B193D2}"/>
+    <workbookView xWindow="14380" yWindow="620" windowWidth="14420" windowHeight="15820" activeTab="2" xr2:uid="{0A9E637F-422C-BE40-81DF-DED3F7B193D2}"/>
   </bookViews>
   <sheets>
     <sheet name="indicator_artstart" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet2" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">indicator_artstart!$A$1:$Y$1207</definedName>
   </definedNames>
-  <calcPr calcId="191029" calcCompleted="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{79F54976-1DA5-4618-B147-4CDE4B953A38}">
       <x14:workbookPr/>
@@ -936,12 +937,13 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="9" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="167" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1067,7 +1069,7 @@
             <xdr:cNvPr id="2051" name="Comment 3" hidden="1">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{706079A3-6B1E-4428-B605-29BE2DBB932F}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{306E483C-D25D-7EC0-7FC5-C54F9040D908}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -1175,7 +1177,7 @@
             <xdr:cNvPr id="2052" name="Comment 4" hidden="1">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DB53D83D-75EE-93CE-42D1-8FFF8B8DA461}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D86766DA-3C20-E7DE-00F6-3143CED42E3B}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -94803,4 +94805,66 @@
     </mc:Choice>
   </mc:AlternateContent>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A641945-2B78-CA4B-848A-AF36F2150087}">
+  <dimension ref="A3:E15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3" s="5">
+        <v>12</v>
+      </c>
+      <c r="B3">
+        <v>16.600000000000001</v>
+      </c>
+      <c r="C3">
+        <f>12/18</f>
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="E3">
+        <f>B3*C3+B4*C4+B5*C5</f>
+        <v>20.355555555555558</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>4</v>
+      </c>
+      <c r="B4">
+        <v>25.1</v>
+      </c>
+      <c r="C4">
+        <f>4/18</f>
+        <v>0.22222222222222221</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>2</v>
+      </c>
+      <c r="B5">
+        <v>33.4</v>
+      </c>
+      <c r="C5">
+        <f>2/18</f>
+        <v>0.1111111111111111</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <f>SUM(A3:A5)</f>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="C15">
+        <f>25/26*1+1/26*5.6</f>
+        <v>1.176923076923077</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Some parameter updates and incoporation
</commit_message>
<xml_diff>
--- a/data/tier_app/iedea_indicators/indicator_artstart.xlsx
+++ b/data/tier_app/iedea_indicators/indicator_artstart.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2ae90f5cbd0fd171/AMC/HIV Prioritization tool/HIV_prioritization_tool/data/tier_app/iedea_indicators/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{5F580FA2-E213-384C-BADC-BD5F5FA04472}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:8_{B0A6AFE0-BE74-AA47-B92B-A74271824EE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14380" yWindow="620" windowWidth="14420" windowHeight="15820" activeTab="2" xr2:uid="{0A9E637F-422C-BE40-81DF-DED3F7B193D2}"/>
+    <workbookView xWindow="3600" yWindow="620" windowWidth="25200" windowHeight="15820" xr2:uid="{0A9E637F-422C-BE40-81DF-DED3F7B193D2}"/>
   </bookViews>
   <sheets>
     <sheet name="indicator_artstart" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">indicator_artstart!$A$1:$Y$1207</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" calcCompleted="0"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{79F54976-1DA5-4618-B147-4CDE4B953A38}">
       <x14:workbookPr/>
@@ -46,7 +46,7 @@
     <author>Leigh Johnson</author>
   </authors>
   <commentList>
-    <comment ref="A45" authorId="0" shapeId="2051" xr:uid="{C7F5560C-5891-0D4A-8B02-151CE51B31CA}">
+    <comment ref="A45" authorId="0" shapeId="1025" xr:uid="{C7F5560C-5891-0D4A-8B02-151CE51B31CA}">
       <text>
         <r>
           <rPr>
@@ -91,7 +91,7 @@
         </mc:Fallback>
       </mc:AlternateContent>
     </comment>
-    <comment ref="A51" authorId="0" shapeId="2052" xr:uid="{68A8BE86-5723-0548-9CD5-6D29C09EDB43}">
+    <comment ref="A51" authorId="0" shapeId="1026" xr:uid="{68A8BE86-5723-0548-9CD5-6D29C09EDB43}">
       <text>
         <r>
           <rPr>
@@ -421,7 +421,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="167" formatCode="0.0000"/>
+    <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
   <fonts count="24" x14ac:knownFonts="1">
     <font>
@@ -942,7 +942,7 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="9" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="167" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
@@ -1066,10 +1066,10 @@
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
-            <xdr:cNvPr id="2051" name="Comment 3" hidden="1">
+            <xdr:cNvPr id="1025" name="Comment 3" hidden="1">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{306E483C-D25D-7EC0-7FC5-C54F9040D908}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{34E42FC4-1DA5-3219-481E-ED143F2E6627}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -1174,10 +1174,10 @@
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
-            <xdr:cNvPr id="2052" name="Comment 4" hidden="1">
+            <xdr:cNvPr id="1026" name="Comment 4" hidden="1">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D86766DA-3C20-E7DE-00F6-3143CED42E3B}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9A0B0DD0-5EDC-CA99-A4C4-94E568AB26C9}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -1587,6 +1587,9 @@
   <sheetPr filterMode="1"/>
   <dimension ref="A1:Y1207"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="21" max="21" width="17" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
@@ -94640,7 +94643,7 @@
       </c>
       <c r="K48" s="4"/>
       <c r="L48" s="4">
-        <f t="shared" ref="L48:L55" si="3">G48*$E$19+H48*$E$18+I48*$E$17</f>
+        <f t="shared" ref="L48:L54" si="3">G48*$E$19+H48*$E$18+I48*$E$17</f>
         <v>6.288732191682256E-3</v>
       </c>
       <c r="M48" s="4"/>

</xml_diff>

<commit_message>
Update sexually active fraction
</commit_message>
<xml_diff>
--- a/data/tier_app/iedea_indicators/indicator_artstart.xlsx
+++ b/data/tier_app/iedea_indicators/indicator_artstart.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:8_{862FEDA9-2982-A447-BBAE-20D444768AFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3600" yWindow="620" windowWidth="25200" windowHeight="15820" activeTab="1" xr2:uid="{0A9E637F-422C-BE40-81DF-DED3F7B193D2}"/>
+    <workbookView xWindow="3600" yWindow="600" windowWidth="25200" windowHeight="15620" activeTab="1" xr2:uid="{0A9E637F-422C-BE40-81DF-DED3F7B193D2}"/>
   </bookViews>
   <sheets>
     <sheet name="indicator_artstart" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">indicator_artstart!$A$1:$Y$1207</definedName>
   </definedNames>
-  <calcPr calcId="191029" calcCompleted="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{79F54976-1DA5-4618-B147-4CDE4B953A38}">
       <x14:workbookPr/>
@@ -1072,7 +1072,7 @@
             <xdr:cNvPr id="1025" name="Comment 3" hidden="1">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{993E2EB2-6D96-FF91-F465-6ED5BE59539C}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D55D4E11-D341-F9E7-B3A7-2A96B7130C48}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -1180,7 +1180,7 @@
             <xdr:cNvPr id="1026" name="Comment 4" hidden="1">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AA741281-279F-845B-F180-4D433DEF459C}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E9210204-5EF6-3BA3-51CD-6043895D201C}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>

</xml_diff>

<commit_message>
Before big mortality supression  shifts
</commit_message>
<xml_diff>
--- a/data/tier_app/iedea_indicators/indicator_artstart.xlsx
+++ b/data/tier_app/iedea_indicators/indicator_artstart.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2ae90f5cbd0fd171/AMC/HIV Prioritization tool/HIV_prioritization_tool/data/tier_app/iedea_indicators/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:8_{862FEDA9-2982-A447-BBAE-20D444768AFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:8_{5CF38630-15AC-1345-8CCD-A3F3D5527AAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3600" yWindow="600" windowWidth="25200" windowHeight="15620" activeTab="1" xr2:uid="{0A9E637F-422C-BE40-81DF-DED3F7B193D2}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15620" activeTab="1" xr2:uid="{0A9E637F-422C-BE40-81DF-DED3F7B193D2}"/>
   </bookViews>
   <sheets>
     <sheet name="indicator_artstart" sheetId="1" r:id="rId1"/>
@@ -46,7 +46,7 @@
     <author>Leigh Johnson</author>
   </authors>
   <commentList>
-    <comment ref="A45" authorId="0" shapeId="1025" xr:uid="{C7F5560C-5891-0D4A-8B02-151CE51B31CA}">
+    <comment ref="A49" authorId="0" shapeId="1025" xr:uid="{C7F5560C-5891-0D4A-8B02-151CE51B31CA}">
       <text>
         <r>
           <rPr>
@@ -77,21 +77,21 @@
               <from>
                 <xdr:col>1</xdr:col>
                 <xdr:colOff>190500</xdr:colOff>
-                <xdr:row>43</xdr:row>
-                <xdr:rowOff>76200</xdr:rowOff>
+                <xdr:row>47</xdr:row>
+                <xdr:rowOff>0</xdr:rowOff>
               </from>
               <to>
                 <xdr:col>2</xdr:col>
                 <xdr:colOff>711200</xdr:colOff>
-                <xdr:row>46</xdr:row>
-                <xdr:rowOff>190500</xdr:rowOff>
+                <xdr:row>50</xdr:row>
+                <xdr:rowOff>114300</xdr:rowOff>
               </to>
             </anchor>
           </commentPr>
         </mc:Fallback>
       </mc:AlternateContent>
     </comment>
-    <comment ref="A51" authorId="0" shapeId="1026" xr:uid="{68A8BE86-5723-0548-9CD5-6D29C09EDB43}">
+    <comment ref="A55" authorId="0" shapeId="1026" xr:uid="{68A8BE86-5723-0548-9CD5-6D29C09EDB43}">
       <text>
         <r>
           <rPr>
@@ -122,14 +122,14 @@
               <from>
                 <xdr:col>1</xdr:col>
                 <xdr:colOff>190500</xdr:colOff>
-                <xdr:row>49</xdr:row>
-                <xdr:rowOff>76200</xdr:rowOff>
+                <xdr:row>53</xdr:row>
+                <xdr:rowOff>0</xdr:rowOff>
               </from>
               <to>
                 <xdr:col>2</xdr:col>
                 <xdr:colOff>711200</xdr:colOff>
-                <xdr:row>52</xdr:row>
-                <xdr:rowOff>190500</xdr:rowOff>
+                <xdr:row>56</xdr:row>
+                <xdr:rowOff>114300</xdr:rowOff>
               </to>
             </anchor>
           </commentPr>
@@ -141,7 +141,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="5097" uniqueCount="85">
+<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="5102" uniqueCount="86">
   <si>
     <t>Region</t>
   </si>
@@ -368,9 +368,6 @@
     <t>Prop 350+</t>
   </si>
   <si>
-    <t>Thembisa mortality</t>
-  </si>
-  <si>
     <t>CD4 stage at ART initiation</t>
   </si>
   <si>
@@ -410,13 +407,19 @@
     <t>Annual HIV mortality rate after first 42 months of ART, females</t>
   </si>
   <si>
-    <t>Take 0.0045 for treated suppressed and unsurpressed non-AHD established</t>
+    <t>prop AHD</t>
   </si>
   <si>
-    <t>Untreataed AHD take 0.18 (first 6 months)</t>
+    <t>Thembisa mortality Table 3.1</t>
   </si>
   <si>
-    <t>prop AHD</t>
+    <t>Mortality in absence of ART</t>
+  </si>
+  <si>
+    <t>Average mortality across cd4 (200+), sex and for 7+ months on ART</t>
+  </si>
+  <si>
+    <t>Take 0.0051 for treated</t>
   </si>
 </sst>
 </file>
@@ -426,7 +429,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="24" x14ac:knownFonts="1">
+  <fonts count="25" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -597,6 +600,12 @@
       <color indexed="81"/>
       <name val="Tahoma"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF1B1B1B"/>
+      <name val="Cambria"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="33">
@@ -940,13 +949,14 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="9" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1058,21 +1068,21 @@
         <xdr:from>
           <xdr:col>1</xdr:col>
           <xdr:colOff>190500</xdr:colOff>
-          <xdr:row>43</xdr:row>
-          <xdr:rowOff>76200</xdr:rowOff>
+          <xdr:row>47</xdr:row>
+          <xdr:rowOff>0</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>2</xdr:col>
           <xdr:colOff>711200</xdr:colOff>
-          <xdr:row>46</xdr:row>
-          <xdr:rowOff>190500</xdr:rowOff>
+          <xdr:row>50</xdr:row>
+          <xdr:rowOff>114300</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="1025" name="Comment 3" hidden="1">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D55D4E11-D341-F9E7-B3A7-2A96B7130C48}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8F2A07FF-57D3-0802-8451-B585FDBEF007}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -1082,7 +1092,7 @@
           </xdr:nvSpPr>
           <xdr:spPr bwMode="auto">
             <a:xfrm>
-              <a:off x="1016000" y="9601200"/>
+              <a:off x="1016000" y="10414000"/>
               <a:ext cx="1346200" cy="723900"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -1166,21 +1176,21 @@
         <xdr:from>
           <xdr:col>1</xdr:col>
           <xdr:colOff>190500</xdr:colOff>
-          <xdr:row>49</xdr:row>
-          <xdr:rowOff>76200</xdr:rowOff>
+          <xdr:row>53</xdr:row>
+          <xdr:rowOff>0</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>2</xdr:col>
           <xdr:colOff>711200</xdr:colOff>
-          <xdr:row>52</xdr:row>
-          <xdr:rowOff>190500</xdr:rowOff>
+          <xdr:row>56</xdr:row>
+          <xdr:rowOff>114300</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="1026" name="Comment 4" hidden="1">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E9210204-5EF6-3BA3-51CD-6043895D201C}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{80F38937-C82B-7D6F-E88B-C0E8D6A4E690}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -1190,7 +1200,7 @@
           </xdr:nvSpPr>
           <xdr:spPr bwMode="auto">
             <a:xfrm>
-              <a:off x="1016000" y="10820400"/>
+              <a:off x="1016000" y="11633200"/>
               <a:ext cx="1346200" cy="723900"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -93996,7 +94006,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:xdr="http://purl.oclc.org/ooxml/drawingml/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C7501CA-F35A-1449-8DEB-8BD038E5B763}">
-  <dimension ref="A1:N55"/>
+  <dimension ref="A1:R60"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.2">
@@ -94088,7 +94098,7 @@
         <v>384</v>
       </c>
       <c r="K3" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="L3">
         <f>E7/I7</f>
@@ -94411,7 +94421,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="33" spans="1:14" ht="22" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:13" ht="22" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>54</v>
       </c>
@@ -94443,7 +94453,7 @@
         <v>7.5977202301903499E-3</v>
       </c>
     </row>
-    <row r="34" spans="1:14" ht="22" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:13" ht="22" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>55</v>
       </c>
@@ -94471,7 +94481,7 @@
         <v>4.5500000000000006E-2</v>
       </c>
     </row>
-    <row r="35" spans="1:14" ht="22" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:13" ht="22" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>56</v>
       </c>
@@ -94493,7 +94503,7 @@
       </c>
       <c r="H35" s="1"/>
     </row>
-    <row r="36" spans="1:14" ht="22" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:13" ht="22" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>57</v>
       </c>
@@ -94514,7 +94524,7 @@
         <v>0.19625000000000004</v>
       </c>
     </row>
-    <row r="37" spans="1:14" ht="22" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:13" ht="22" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>58</v>
       </c>
@@ -94535,7 +94545,7 @@
         <v>0.50600000000000001</v>
       </c>
     </row>
-    <row r="38" spans="1:14" ht="22" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:13" ht="22" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>59</v>
       </c>
@@ -94556,280 +94566,346 @@
         <v>1.3062499999999999</v>
       </c>
     </row>
-    <row r="41" spans="1:14" ht="22" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:13" ht="22" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="42" spans="1:13" ht="22" x14ac:dyDescent="0.25">
+      <c r="A42" s="1"/>
+    </row>
+    <row r="43" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A43" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="44" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A44" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="45" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A45" s="6">
+        <v>0</v>
+      </c>
+      <c r="B45">
+        <v>0</v>
+      </c>
+      <c r="C45">
+        <v>3.3000000000000002E-2</v>
+      </c>
+      <c r="D45">
+        <v>0.254</v>
+      </c>
+    </row>
+    <row r="47" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A47" s="2"/>
+      <c r="G47" s="3" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A43" s="2"/>
-      <c r="G43" s="3" t="s">
+    <row r="48" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A48" s="2"/>
+      <c r="G48" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="H48" s="2" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A44" s="2"/>
-      <c r="G44" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="H44" s="2" t="s">
+      <c r="I48" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="I44" s="2" t="s">
+      <c r="J48" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="K48" s="2"/>
+      <c r="L48" s="2"/>
+      <c r="M48" s="2"/>
+    </row>
+    <row r="49" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A49" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="J44" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="K44" s="2"/>
-      <c r="L44" s="2"/>
-      <c r="M44" s="2"/>
-    </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A45" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="G45" s="4">
+      <c r="G49" s="4">
         <v>2.0000000000000001E-4</v>
       </c>
-      <c r="H45" s="4">
+      <c r="H49" s="4">
         <v>1.6000000000000001E-3</v>
       </c>
-      <c r="I45" s="4">
+      <c r="I49" s="4">
         <v>1.46E-2</v>
       </c>
-      <c r="J45" s="4">
-        <v>0.21679999999999999</v>
-      </c>
-      <c r="K45" s="4"/>
-      <c r="L45" s="4">
-        <f>G45*E19+H45*E18+I45*E17</f>
-        <v>5.6079148078860266E-3</v>
-      </c>
-      <c r="M45" s="4"/>
-      <c r="N45" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A46" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="G46" s="4">
-        <v>8.9999999999999998E-4</v>
-      </c>
-      <c r="H46" s="4">
-        <v>5.0000000000000001E-3</v>
-      </c>
-      <c r="I46" s="4">
-        <v>1.32E-2</v>
-      </c>
-      <c r="J46" s="4">
-        <v>5.33E-2</v>
-      </c>
-      <c r="K46" s="4"/>
-      <c r="L46" s="4">
-        <f>G46*$E$19+H46*$E$18+I46*$E$17</f>
-        <v>6.2874082601813205E-3</v>
-      </c>
-      <c r="M46" s="4"/>
-    </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A47" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="G47" s="4">
-        <v>2.7000000000000001E-3</v>
-      </c>
-      <c r="H47" s="4">
-        <v>8.5000000000000006E-3</v>
-      </c>
-      <c r="I47" s="4">
-        <v>1.1599999999999999E-2</v>
-      </c>
-      <c r="J47" s="4">
-        <v>2.81E-2</v>
-      </c>
-      <c r="K47" s="4"/>
-      <c r="L47" s="4">
-        <f>G47*$E$19+H47*$E$18+I47*$E$17</f>
-        <v>7.3476183623542952E-3</v>
-      </c>
-      <c r="M47" s="4"/>
-    </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A48" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="G48" s="4">
-        <v>4.1999999999999997E-3</v>
-      </c>
-      <c r="H48" s="4">
-        <v>7.6E-3</v>
-      </c>
-      <c r="I48" s="4">
-        <v>7.6E-3</v>
-      </c>
-      <c r="J48" s="4">
-        <v>1.8499999999999999E-2</v>
-      </c>
-      <c r="K48" s="4"/>
-      <c r="L48" s="4">
-        <f t="shared" ref="L48:L54" si="4">G48*$E$19+H48*$E$18+I48*$E$17</f>
-        <v>6.288732191682256E-3</v>
-      </c>
-      <c r="M48" s="4"/>
-    </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A49" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="G49" s="4">
-        <v>4.8999999999999998E-3</v>
-      </c>
-      <c r="H49" s="4">
-        <v>6.3E-3</v>
-      </c>
-      <c r="I49" s="4">
-        <v>6.3E-3</v>
-      </c>
       <c r="J49" s="4">
-        <v>1.52E-2</v>
+        <v>0.25540000000000002</v>
       </c>
       <c r="K49" s="4"/>
       <c r="L49" s="4">
-        <f t="shared" si="4"/>
-        <v>5.7600661965750474E-3</v>
+        <f>G49*E19+H49*E18+I49*E17</f>
+        <v>5.6079148078860266E-3</v>
       </c>
       <c r="M49" s="4"/>
-      <c r="N49" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A50" s="2"/>
-      <c r="G50" s="4"/>
-      <c r="H50" s="4"/>
-      <c r="I50" s="4"/>
-      <c r="J50" s="4"/>
+    </row>
+    <row r="50" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A50" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="G50" s="4">
+        <v>8.9999999999999998E-4</v>
+      </c>
+      <c r="H50" s="4">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="I50" s="4">
+        <v>1.32E-2</v>
+      </c>
+      <c r="J50" s="4">
+        <v>6.13E-2</v>
+      </c>
       <c r="K50" s="4"/>
-      <c r="L50" s="4"/>
+      <c r="L50" s="4">
+        <f>G50*$E$19+H50*$E$18+I50*$E$17</f>
+        <v>6.2874082601813205E-3</v>
+      </c>
       <c r="M50" s="4"/>
     </row>
-    <row r="51" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A51" s="2" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="G51" s="4">
-        <v>1E-4</v>
+        <v>2.7000000000000001E-3</v>
       </c>
       <c r="H51" s="4">
-        <v>1.6000000000000001E-3</v>
+        <v>8.5000000000000006E-3</v>
       </c>
       <c r="I51" s="4">
-        <v>1.5900000000000001E-2</v>
+        <v>1.1599999999999999E-2</v>
       </c>
       <c r="J51" s="4">
-        <v>0.1699</v>
+        <v>3.0599999999999999E-2</v>
       </c>
       <c r="K51" s="4"/>
       <c r="L51" s="4">
-        <f t="shared" si="4"/>
-        <v>6.0241329687724856E-3</v>
+        <f>G51*$E$19+H51*$E$18+I51*$E$17</f>
+        <v>7.3476183623542952E-3</v>
       </c>
       <c r="M51" s="4"/>
     </row>
-    <row r="52" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A52" s="2" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="G52" s="4">
-        <v>8.0000000000000004E-4</v>
+        <v>4.1999999999999997E-3</v>
       </c>
       <c r="H52" s="4">
-        <v>4.4999999999999997E-3</v>
+        <v>7.6E-3</v>
       </c>
       <c r="I52" s="4">
-        <v>1.01E-2</v>
+        <v>7.6E-3</v>
       </c>
       <c r="J52" s="4">
-        <v>4.1599999999999998E-2</v>
+        <v>2.0199999999999999E-2</v>
       </c>
       <c r="K52" s="4"/>
       <c r="L52" s="4">
-        <f t="shared" si="4"/>
-        <v>5.0321053388976827E-3</v>
+        <f t="shared" ref="L52:L58" si="4">G52*$E$19+H52*$E$18+I52*$E$17</f>
+        <v>6.288732191682256E-3</v>
       </c>
       <c r="M52" s="4"/>
     </row>
-    <row r="53" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A53" s="2" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="G53" s="4">
-        <v>2E-3</v>
+        <v>4.8999999999999998E-3</v>
       </c>
       <c r="H53" s="4">
-        <v>5.7000000000000002E-3</v>
+        <v>6.3E-3</v>
       </c>
       <c r="I53" s="4">
-        <v>5.7000000000000002E-3</v>
+        <v>6.3E-3</v>
       </c>
       <c r="J53" s="4">
-        <v>2.1600000000000001E-2</v>
+        <v>1.66E-2</v>
       </c>
       <c r="K53" s="4"/>
       <c r="L53" s="4">
         <f t="shared" si="4"/>
+        <v>5.7600661965750474E-3</v>
+      </c>
+      <c r="M53" s="4"/>
+    </row>
+    <row r="54" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A54" s="2"/>
+      <c r="G54" s="4"/>
+      <c r="H54" s="4"/>
+      <c r="I54" s="4"/>
+      <c r="J54" s="4"/>
+      <c r="K54" s="4"/>
+      <c r="L54" s="4"/>
+      <c r="M54" s="4"/>
+    </row>
+    <row r="55" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A55" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="G55" s="4">
+        <v>1E-4</v>
+      </c>
+      <c r="H55" s="4">
+        <v>1.6000000000000001E-3</v>
+      </c>
+      <c r="I55" s="4">
+        <v>1.5900000000000001E-2</v>
+      </c>
+      <c r="J55" s="4">
+        <v>0.2072</v>
+      </c>
+      <c r="K55" s="4"/>
+      <c r="L55" s="4">
+        <f t="shared" si="4"/>
+        <v>6.0241329687724856E-3</v>
+      </c>
+      <c r="M55" s="4"/>
+    </row>
+    <row r="56" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A56" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="G56" s="4">
+        <v>8.0000000000000004E-4</v>
+      </c>
+      <c r="H56" s="4">
+        <v>4.4999999999999997E-3</v>
+      </c>
+      <c r="I56" s="4">
+        <v>1.01E-2</v>
+      </c>
+      <c r="J56" s="4">
+        <v>4.9000000000000002E-2</v>
+      </c>
+      <c r="K56" s="4"/>
+      <c r="L56" s="4">
+        <f t="shared" si="4"/>
+        <v>5.0321053388976827E-3</v>
+      </c>
+      <c r="M56" s="4"/>
+      <c r="O56" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="57" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A57" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="G57" s="4">
+        <v>2E-3</v>
+      </c>
+      <c r="H57" s="4">
+        <v>5.7000000000000002E-3</v>
+      </c>
+      <c r="I57" s="4">
+        <v>5.7000000000000002E-3</v>
+      </c>
+      <c r="J57" s="4">
+        <v>2.35E-2</v>
+      </c>
+      <c r="K57" s="4"/>
+      <c r="L57" s="4">
+        <f t="shared" si="4"/>
         <v>4.2730320909483378E-3</v>
       </c>
-      <c r="M53" s="4"/>
-    </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A54" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="G54" s="4">
+      <c r="M57" s="4"/>
+      <c r="O57">
+        <v>6.2874082601813205E-3</v>
+      </c>
+      <c r="P57">
+        <v>5.0321053388976827E-3</v>
+      </c>
+      <c r="R57">
+        <f>AVERAGE(O57:P60)</f>
+        <v>5.077374442365808E-3</v>
+      </c>
+    </row>
+    <row r="58" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A58" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="G58" s="4">
         <v>2.7000000000000001E-3</v>
       </c>
-      <c r="H54" s="4">
+      <c r="H58" s="4">
         <v>3.3999999999999998E-3</v>
       </c>
-      <c r="I54" s="4">
+      <c r="I58" s="4">
         <v>3.3999999999999998E-3</v>
       </c>
-      <c r="J54" s="4">
-        <v>1.2999999999999999E-2</v>
-      </c>
-      <c r="K54" s="4"/>
-      <c r="L54" s="4">
+      <c r="J58" s="4">
+        <v>1.41E-2</v>
+      </c>
+      <c r="K58" s="4"/>
+      <c r="L58" s="4">
         <f t="shared" si="4"/>
         <v>3.130033098287523E-3</v>
       </c>
-      <c r="M54" s="4"/>
-    </row>
-    <row r="55" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A55" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="G55" s="4">
+      <c r="M58" s="4"/>
+      <c r="O58">
+        <v>7.3476183623542952E-3</v>
+      </c>
+      <c r="P58">
+        <v>4.2730320909483378E-3</v>
+      </c>
+    </row>
+    <row r="59" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A59" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="G59" s="4">
         <v>2.5000000000000001E-3</v>
       </c>
-      <c r="H55" s="4">
+      <c r="H59" s="4">
         <v>2.5000000000000001E-3</v>
       </c>
-      <c r="I55" s="4">
+      <c r="I59" s="4">
         <v>2.5000000000000001E-3</v>
       </c>
-      <c r="J55" s="4">
-        <v>9.4000000000000004E-3</v>
-      </c>
-      <c r="K55" s="4"/>
-      <c r="L55" s="4">
-        <f>G55*$E$19+H55*$E$18+I55*$E$17</f>
+      <c r="J59" s="4">
+        <v>1.03E-2</v>
+      </c>
+      <c r="K59" s="4"/>
+      <c r="L59" s="4">
+        <f>G59*$E$19+H59*$E$18+I59*$E$17</f>
         <v>2.5000000000000001E-3</v>
       </c>
-      <c r="M55" s="4"/>
+      <c r="M59" s="4"/>
+      <c r="O59">
+        <v>6.288732191682256E-3</v>
+      </c>
+      <c r="P59">
+        <v>3.130033098287523E-3</v>
+      </c>
+      <c r="R59" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="60" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="O60">
+        <v>5.7600661965750474E-3</v>
+      </c>
+      <c r="P60">
+        <v>2.5000000000000001E-3</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Additional mortality split for new AHD vs established AHD
</commit_message>
<xml_diff>
--- a/data/tier_app/iedea_indicators/indicator_artstart.xlsx
+++ b/data/tier_app/iedea_indicators/indicator_artstart.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2ae90f5cbd0fd171/AMC/HIV Prioritization tool/HIV_prioritization_tool/data/tier_app/iedea_indicators/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:8_{5CF38630-15AC-1345-8CCD-A3F3D5527AAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:8_{904189FE-831A-5E46-8F0E-07FFC11D5674}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15620" activeTab="1" xr2:uid="{0A9E637F-422C-BE40-81DF-DED3F7B193D2}"/>
+    <workbookView xWindow="-32160" yWindow="-800" windowWidth="28800" windowHeight="15620" activeTab="1" xr2:uid="{0A9E637F-422C-BE40-81DF-DED3F7B193D2}"/>
   </bookViews>
   <sheets>
     <sheet name="indicator_artstart" sheetId="1" r:id="rId1"/>
@@ -141,7 +141,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="5102" uniqueCount="86">
+<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="5103" uniqueCount="86">
   <si>
     <t>Region</t>
   </si>
@@ -1082,7 +1082,7 @@
             <xdr:cNvPr id="1025" name="Comment 3" hidden="1">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8F2A07FF-57D3-0802-8451-B585FDBEF007}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5125D315-E02E-A254-96A9-5059FBDB559D}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -1190,7 +1190,7 @@
             <xdr:cNvPr id="1026" name="Comment 4" hidden="1">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{80F38937-C82B-7D6F-E88B-C0E8D6A4E690}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4A3935F0-FB14-32E6-3EA3-11A643D2B8F7}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -94653,6 +94653,9 @@
         <v>5.6079148078860266E-3</v>
       </c>
       <c r="M49" s="4"/>
+      <c r="O49" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="50" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A50" s="2" t="s">
@@ -94676,6 +94679,16 @@
         <v>6.2874082601813205E-3</v>
       </c>
       <c r="M50" s="4"/>
+      <c r="O50">
+        <v>6.13E-2</v>
+      </c>
+      <c r="P50">
+        <v>4.9000000000000002E-2</v>
+      </c>
+      <c r="Q50">
+        <f>AVERAGE(O50:P53)</f>
+        <v>2.8199999999999999E-2</v>
+      </c>
     </row>
     <row r="51" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A51" s="2" t="s">
@@ -94699,6 +94712,12 @@
         <v>7.3476183623542952E-3</v>
       </c>
       <c r="M51" s="4"/>
+      <c r="O51">
+        <v>3.0599999999999999E-2</v>
+      </c>
+      <c r="P51">
+        <v>2.35E-2</v>
+      </c>
     </row>
     <row r="52" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A52" s="2" t="s">
@@ -94722,6 +94741,12 @@
         <v>6.288732191682256E-3</v>
       </c>
       <c r="M52" s="4"/>
+      <c r="O52">
+        <v>2.0199999999999999E-2</v>
+      </c>
+      <c r="P52">
+        <v>1.41E-2</v>
+      </c>
     </row>
     <row r="53" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A53" s="2" t="s">
@@ -94745,6 +94770,12 @@
         <v>5.7600661965750474E-3</v>
       </c>
       <c r="M53" s="4"/>
+      <c r="O53">
+        <v>1.66E-2</v>
+      </c>
+      <c r="P53">
+        <v>1.03E-2</v>
+      </c>
     </row>
     <row r="54" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A54" s="2"/>

</xml_diff>

<commit_message>
Re-do of unit tests
</commit_message>
<xml_diff>
--- a/data/tier_app/iedea_indicators/indicator_artstart.xlsx
+++ b/data/tier_app/iedea_indicators/indicator_artstart.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2ae90f5cbd0fd171/AMC/HIV Prioritization tool/HIV_prioritization_tool/data/tier_app/iedea_indicators/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:8_{904189FE-831A-5E46-8F0E-07FFC11D5674}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:8_{D3F947EA-9C98-4A49-B715-296C9B83E97D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-32160" yWindow="-800" windowWidth="28800" windowHeight="15620" activeTab="1" xr2:uid="{0A9E637F-422C-BE40-81DF-DED3F7B193D2}"/>
   </bookViews>
@@ -1082,7 +1082,7 @@
             <xdr:cNvPr id="1025" name="Comment 3" hidden="1">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5125D315-E02E-A254-96A9-5059FBDB559D}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{340EFB73-13D1-CE32-34C0-3F01BC29EF48}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -1190,7 +1190,7 @@
             <xdr:cNvPr id="1026" name="Comment 4" hidden="1">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4A3935F0-FB14-32E6-3EA3-11A643D2B8F7}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{93E23905-E076-48B6-DDCA-7C1521DAF0B4}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>

</xml_diff>